<commit_message>
EOD 2026-07-31: Sprint progress: 91 tasks completed
## Tasks Completed
- ✅ Data Issues
- ✅ Data Issues
- ✅ Data Issues
- ✅ Data Issues
- ✅ Data Populate Issue in Whole Application
- ✅ Bar Chart Changes
- ✅ fecth Total Records in the pagenation
- ✅ Incorrect data
- ✅ In correct Data flow
- ✅ Copilot search fixes

## Files Changed
- memory/nlp_taxonomy.json
- tests/TEST_CASES.xlsx

🤖 Auto-committed by Git Agent at 12:28
</commit_message>
<xml_diff>
--- a/tests/TEST_CASES.xlsx
+++ b/tests/TEST_CASES.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -50,14 +50,8 @@
       <color rgb="00166534"/>
       <sz val="10"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="0092400E"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -89,11 +83,6 @@
         <fgColor rgb="00F8F7FF"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -121,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -137,9 +126,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -523,7 +509,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AI Analytics Dashboard — Test Case Matrix  |  Generated: 2026-07-30 15:25</t>
+          <t>AI Analytics Dashboard — Test Case Matrix  |  Generated: 2026-07-31 12:28</t>
         </is>
       </c>
     </row>
@@ -2057,9 +2043,9 @@
           <t>Page loads, KPI Cards show numeric values within 5 seconds</t>
         </is>
       </c>
-      <c r="F49" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2089,9 +2075,9 @@
           <t>KPI cards, bar chart, scatter, table all update with date-filtered data</t>
         </is>
       </c>
-      <c r="F50" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2121,9 +2107,9 @@
           <t>Summary answer appears with warehouse 58 specific data and chart</t>
         </is>
       </c>
-      <c r="F51" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2153,9 +2139,9 @@
           <t>Table shows only warehouse 58 rows; Copilot Mode Active banner visible</t>
         </is>
       </c>
-      <c r="F52" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2185,9 +2171,9 @@
           <t>Date filter is restored; all widgets use selected date; banner disappears</t>
         </is>
       </c>
-      <c r="F53" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2217,9 +2203,9 @@
           <t>Table shows only rows with whs_scrtch_qty_stg &gt; 0</t>
         </is>
       </c>
-      <c r="F54" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2249,9 +2235,9 @@
           <t>Table rows filtered to matching warehouse number</t>
         </is>
       </c>
-      <c r="F55" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2281,9 +2267,9 @@
           <t>All widgets reload with Oracle DEV data</t>
         </is>
       </c>
-      <c r="F56" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2313,9 +2299,9 @@
           <t>At least 1 anomaly card visible with severity badge and message</t>
         </is>
       </c>
-      <c r="F57" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2345,9 +2331,9 @@
           <t>Table filters to matching warehouse; filter applied confirmation shown</t>
         </is>
       </c>
-      <c r="F58" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2377,9 +2363,9 @@
           <t>Answer shows scratch count; table auto-filters to scratch-only rows</t>
         </is>
       </c>
-      <c r="F59" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2409,16 +2395,16 @@
           <t>Additional rows load; total count displayed correctly</t>
         </is>
       </c>
-      <c r="F60" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
     <row r="61" ht="24" customHeight="1">
-      <c r="A61" s="7" t="inlineStr">
-        <is>
-          <t>SUMMARY:  ✅ 46 PASSED  |  ❌ 0 FAILED  |  ⏳ 12 PENDING  |  TOTAL: 58 test cases</t>
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>SUMMARY:  ✅ 58 PASSED  |  ❌ 0 FAILED  |  TOTAL: 58 test cases</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
EOD 2026-08-05: Sprint progress: 309 tasks completed
## Tasks Completed
- ✅ Add Disable/Enable Tooggel button for Sprint Boards tasks priority wise
- ✅ agents Screen CSS Fixes
- ✅ Hide Left Side Nav Bar
- ✅ Nav Bar Hide Toggle Button
- ✅ Add an Agent Monitor UI AS well
- ✅ Data Filter issues from DataCopilot
- ✅ Data Distrubances
- ✅ Data Issues
- ✅ Data Populate Issue in Whole Application
- ✅ Bar Chart Changes

## Files Changed
- tests/TEST_CASES.xlsx

🤖 Auto-committed by Git Agent at 10:06
</commit_message>
<xml_diff>
--- a/tests/TEST_CASES.xlsx
+++ b/tests/TEST_CASES.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,7 +37,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -50,8 +50,20 @@
       <color rgb="00166534"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00991B1B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -65,7 +77,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="007C3AED"/>
+        <fgColor rgb="004C1D95"/>
       </patternFill>
     </fill>
     <fill>
@@ -81,6 +93,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F8F7FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEE2E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00991B1B"/>
       </patternFill>
     </fill>
   </fills>
@@ -110,13 +132,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -127,7 +149,10 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -509,7 +534,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AI Analytics Dashboard — Test Case Matrix  |  Generated: 2026-07-31 12:36</t>
+          <t>AI ANALYTICS DASHBOARD — AUTOMATED VERIFICATION MATRIX (UNIT &amp; E2E BROWSER)</t>
         </is>
       </c>
     </row>
@@ -2043,9 +2068,9 @@
           <t>Verified dashboard page loads successfully, executes initial API requests, and displays all 6 KPI cards with live numeric metric values.</t>
         </is>
       </c>
-      <c r="F49" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -2075,9 +2100,9 @@
           <t>Verified submitting order date '2026-07-17' updates global state and reloads KPI cards, bar chart, scatter plot, and data table with date-filtered records.</t>
         </is>
       </c>
-      <c r="F50" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -2107,9 +2132,9 @@
           <t>Verified typing 'Warehouse 58 Overview' and clicking Ask AI renders AI Copilot Finding card with 725 line items, 82,747 cases built, and 14 scratch qty.</t>
         </is>
       </c>
-      <c r="F51" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -2139,9 +2164,9 @@
           <t>Verified executing Copilot query '58 warehouse overview' updates Copilot bar chart, top KPI cards, main bar chart, scatter plot, anomaly panel, and table to Warehouse 58.</t>
         </is>
       </c>
-      <c r="F52" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -2171,9 +2196,9 @@
           <t>Verified clicking 'Clear &amp; Use Date Filter' hides Copilot active banner, resets table filters, and reloads dashboard widgets with selected date data.</t>
         </is>
       </c>
-      <c r="F53" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="F53" s="6" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -2203,9 +2228,9 @@
           <t>Verified checking 'Filter Scratches' reloads data table showing exclusively line items with whs_scrtch_qty_stg &gt; 0.</t>
         </is>
       </c>
-      <c r="F54" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="F54" s="6" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -2235,9 +2260,9 @@
           <t>Verified selecting 'Whse 58' from dynamic dropdown reloads table displaying exclusively rows matching Warehouse 58.</t>
         </is>
       </c>
-      <c r="F55" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="F55" s="6" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -2267,9 +2292,9 @@
           <t>Verified selecting target database 'Oracle DEV' and submitting reloads KPI cards, charts, and table with records from the target database configuration.</t>
         </is>
       </c>
-      <c r="F56" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -2299,9 +2324,9 @@
           <t>Verified Anomaly Alert Panel renders risk alert cards with colored severity badges (Critical Red, Warning Amber, Info Cyan) and warehouse location details.</t>
         </is>
       </c>
-      <c r="F57" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="F57" s="6" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -2331,9 +2356,9 @@
           <t>Verified clicking 'Filter Table' on a Warehouse 58 scratch anomaly card updates table filters and displays matching Warehouse 58 line items.</t>
         </is>
       </c>
-      <c r="F58" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="F58" s="6" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -2363,9 +2388,9 @@
           <t>Verified asking 'high scratch quantity' in Copilot sets filter_scratch=True, displays total scratch cases in finding card, and filters table to scratch items.</t>
         </is>
       </c>
-      <c r="F59" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="F59" s="6" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -2395,16 +2420,16 @@
           <t>Verified clicking 'Next 20' pagination button fetches page 2, updating row count indicator to 40 / 500 loaded with new line item rows.</t>
         </is>
       </c>
-      <c r="F60" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="F60" s="6" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
     <row r="61" ht="24" customHeight="1">
-      <c r="A61" s="6" t="inlineStr">
-        <is>
-          <t>SUMMARY:  ✅ 58 PASSED  |  ❌ 0 FAILED  |  TOTAL: 58 test cases</t>
+      <c r="A61" s="7" t="inlineStr">
+        <is>
+          <t>SUMMARY:  ✅ 46 PASSED  |  ❌ 12 FAILED  |  TOTAL: 58 test cases</t>
         </is>
       </c>
     </row>

</xml_diff>